<commit_message>
114b: METHODS_REVIEW current through Sep 1
Adds four method rows -- ligand-conditioned substitution priors, backbone
envelope vs cavity volume, pose-check MD, RFdiffusion3 motif scaffolding -- and
seven timeline entries covering the audit, the 62a retraction, the decoded
true-negative set, the volume baseline and the donor-ranking reversal.
</commit_message>
<xml_diff>
--- a/data/methods_review.xlsx
+++ b/data/methods_review.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Glossary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Methods'!$A$1:$M$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Methods'!$A$1:$M$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -55,22 +55,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C6E7C6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BFE3F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2D4D4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E7C6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFF0C2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BFE3F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -831,82 +831,166 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Aug 28</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Umbrella sampling FAILS its pre-registered hysteresis test by 15x with a sign flip. The arm is closed.</t>
+          <t>External audit finds the factorial extraction bug; 62a is recomputed on the restored 1.6 us and RETRACTED -- the dF sign flips across replicate pairings.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Aug 28</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Graft direction closed: enlargement is neither insertion (&lt;=3 inserted residues in any donor) nor displacement (sheet-helix r = -0.18).</t>
+          <t>Park's Figure 5 decoded: 7,045 true negatives, the first in the project. AUC 0.868 on mandipropamid.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Aug 28</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Beltran-45, the first held-out benchmark: Tian's frequency prior transfers at 64 % recall, then saturates at the 67 % vocabulary ceiling.</t>
+          <t>Clash relief is not specific: azoxystrobin and lufenuron clash as hard as mandipropamid and have zero responders of 475.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Jannis: the mandipropamid library was built in the FORCED K59R backbone. Every 'K59R is invisible' record was scoring a prediction nobody had to make.</t>
+          <t>The volume baseline, applied retroactively: side-chain volume alone gives 0.781 on mandipropamid, so the whole structural pipeline buys ~0.09.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ddG replicate noise measured: 0.21 REU against a 2.7 REU signal. The score is precise; the shrink-penalty is what makes it wrong.</t>
+          <t>Desolvation reaches fludioxonil (0.682 where the total is 0.550) and then FAILS to transfer to the WIN library.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>DSM doubles enumerated in full (35,863): 4.6x narrowing to a first hit, but A160 found at 2.63x and F159 at exactly chance.</t>
+          <t>Ligand-similarity priors beat the blind bar but the control shows it is lookup; the per-position version fails on data density.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>Sep 1</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Backbone envelope overturns the donor ranking -- 2PCS's polyGly volume equals PYR1's, so its cavity is side chains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Umbrella sampling FAILS its pre-registered hysteresis test by 15x with a sign flip. The arm is closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Graft direction closed: enlargement is neither insertion (&lt;=3 inserted residues in any donor) nor displacement (sheet-helix r = -0.18).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Aug 28</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Beltran-45, the first held-out benchmark: Tian's frequency prior transfers at 64 % recall, then saturates at the 67 % vocabulary ceiling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>Aug 31</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Jannis: the mandipropamid library was built in the FORCED K59R backbone. Every 'K59R is invisible' record was scoring a prediction nobody had to make.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Aug 31</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>ddG replicate noise measured: 0.21 REU against a 2.7 REU signal. The score is precise; the shrink-penalty is what makes it wrong.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Aug 31</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>DSM doubles enumerated in full (35,863): 4.6x narrowing to a first hit, but A160 found at 2.63x and F159 at exactly chance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Aug 31</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>TRUE NEGATIVES INVENTORIED: sd07 has 0, sd09 has 3, sd01 is ligand-level only. Accuracy cannot be measured on the data that exists.</t>
         </is>
@@ -923,7 +1007,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1011,52 +1095,52 @@
     <row r="2" ht="108" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Thermodynamic integration (TI)</t>
+          <t>Ligand-conditioned substitution priors</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Affinity - energetics</t>
+          <t>Design - library</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Alchemical free-energy difference along a lambda path with softcore; two legs give a selectivity ddG.</t>
+          <t>Similarity-weighted priors over substitutions: whole-molecule ECFP4/descriptor aggregation, and a per-pocket-position pharmacophore version.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Asked whether TI can rank PYR1 point mutations well enough to choose between them.</t>
+          <t>Jannis's MSA analogy -- aggregate everything known about every screened ligand to BIAS the choice among sequences other filters allow, rather than to predict.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>PYR1 + ABA / mandipropamid; 85-88, 90-92</t>
+          <t>194 sd03 ligands with clones; 181 with co-folded poses</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Aug 22-24</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>A working Amber TI pipeline with six setup traps documented. The pilot ran 72/72 and the quadruple 48/48. The crystal arm gives the right SIGN and NO CALL at +-2.34 kcal/mol against an effect of ~1.</t>
+          <t>The whole-molecule prior beats the ligand-blind bar by +0.05 recall@20 (0.398 vs 0.345), five times 52's +0.010, and is STABLE across the weighting exponent rather than sitting on a knife edge. Paired: +0.053, t = 17.4, 49 of 50 splits positive.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>The docked arm is structurally invalid -- the ligand collapses into deleted F108's volume, which breaks the whole dock-into-an-enlarged-pocket workflow. The pilot's own error bar was 20x too small until a regex double-counting frames was found.</t>
+          <t>The control kills the MSA analogy: the entire gain comes from ligands WITH a close analog (+0.191 at Tanimoto &gt;= 0.5) and it is NEGATIVE where none exists (-0.036 at &lt; 0.2) -- the case a novel target is in. The per-position version fails at every shell radius and monotonically worse the more local it gets, because the pocket is 11.6 A long so a 7 A shell is the whole molecule, and a 3.5 A shell leaves too few ligands per position.</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>8.3 GPU-days per variant pair is the real cost, which is what moved the project off affinity prediction and onto library enrichment (47).</t>
+          <t>Gate it on max Tanimoto &gt;= 0.25: +0.056 across 69 % of ligands, switched off for novel chemotypes. A data-density limit, not a flaw in the idea -- 18 position-specific priors cannot be estimated from 182 ligands.</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>RETIRED</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -1066,64 +1150,64 @@
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>85-92; jobs 27725295 and predecessors</t>
+          <t>177, 178</t>
         </is>
       </c>
     </row>
     <row r="3" ht="108" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Umbrella sampling of the open/closed coordinate</t>
+          <t>Backbone envelope vs cavity volume</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Conformation - energetics</t>
+          <t>Pocket - structure</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>62 windows along P88 CA - R116 CA with WHAM, forward and reverse seeded, holo and apo.</t>
+          <t>polyGly free volume inside a structurally-aligned wall hull, plus depth and depth/width of that envelope. Never cavity-derived.</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>The last route to the open/closed dG that unbiased MD cannot reach (62), and so to the switching cost of a designed pocket.</t>
+          <t>Jannis: cavity volume conflates backbone with side chains, and if a donor's larger cavity is just smaller side chains that is cheaper to get by mutating PYR1.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>S1/S2/S9/S10 factorial seeds; 1.24 us biased</t>
+          <t>PYR1 + 6 SRPBCC donors + 3 START lipid-transfer domains</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Aug 25-28</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>FAILS its own pre-registered test. Forward and reverse disagree by 3.22 kcal/mol holo and 2.74 apo against a half-split drift bar of 0.22 and 1.05, and the SIGN of the tilt flips between seedings (+4.61 vs -3.29). Calibration also fails on its own terms (ddG -1.90 where a pass needs positive).</t>
+          <t>It overturned the donor ranking. 2PCS -- preferred throughout this project -- has a polyGly volume of 1173 against PYR1's 1184, DEAD EVEN: its 570 A^3 cavity against PYR1's 164 is entirely side chains. Same for 2NS9, 6AWV, 3OQU. The real difference is SHAPE: PYR1's envelope is nearly isotropic (d/w 1.25) while CERT/2E3M is 36.8 A deep at d/w 2.36.</t>
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>My own 70/127 repair destroyed the two-directional seeding, which 81b suspected and 85 confirmed. Separately, the seeds came from only 5 of the 11 finished factorial trajectories (see the extraction bug below).</t>
+          <t>This metric was wrong twice before (143's circular envelope, 143's poly-Gly column reporting a vanished component as 0-3 A^3). 145 fixed both and this uses that version.</t>
         </is>
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>A 15x miss with a sign flip is protocol, not sampling length. Do not rerun. Switch cost is a Y2H question.</t>
+          <t>Since 8's limit on PYR1 is LENGTH not volume, the importable difference is a longer pocket, not a bigger one -- and no donor offers both. Design targets should be depth and d/w.</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>RETIRED</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -1133,64 +1217,64 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>GPU short_gpu</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>111-113, 127, 136, 138; jobs 27854551</t>
+          <t>181, 182</t>
         </is>
       </c>
     </row>
     <row r="4" ht="108" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Boltz-2 co-folding and affinity head</t>
+          <t>Pose-check MD</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Affinity - ML</t>
+          <t>Structure - validation</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Structure + binding prediction from sequence and SMILES; affinity_probability_binary and affinity_pred_value.</t>
+          <t>6 ligand/receptor systems x 3 replicates x 20 ns; ligand heavy-atom RMSD to the starting pose with the protein core superposed.</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Asked three separate questions: can it rank pocket VARIANTS, can it predict ligand TRACTABILITY, and can it supply poses for ligands with no crystal structure.</t>
+          <t>Asks whether MD retains a predicted pose, since most poses this project trains on were predicted once and 93a showed co-folding places a ligand in the pocket regardless of whether it belongs.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>718 sensor structures; 362 property-matched tractability models; 50 pose predictions</t>
+          <t>ABA, mandipropamid (crystal AND predicted), WIN, fludioxonil, benoxacor</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Aug 27-31</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>Variant ranking: NO (within-ligand rho -0.028, and the binder classifier calls 90 % of real sensors non-binders). Poses: it finds the right pocket every time and builds the CLOSED receptor (gate RMSD 1.15-1.80 A), with a single consistent pose for about a quarter of ligands (97 of 362 under 1.0 A).</t>
+          <t>IN FLIGHT, 8 of 18 complete. All six systems built at 39,507-43,893 atoms with no parmchk2 ATTN flags -- no guessed parameters, which matters because a guessed torsion is indistinguishable from a bad pose in an RMSD trace.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Two silent failures cost whole arrays: a single trailing NUL byte in the shared a3m, and a ONE-RESIDUE mismatch between the a3m query and the input sequence, which makes it abandon the MSA and fold single-sequence at pLDDT 49 instead of 96. Neither errors.</t>
+          <t>Six build attempts were needed, every failure a silent format mismatch (explicit hydrogens, sanitize=False, MDL aromatic bond type 4). Recorded in the script so they are not rediscovered.</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>Assert the fold (median pLDDT &gt;= 80) and assert the a3m query equals the input sequence, before any downstream number is computed.</t>
+          <t>Two paired comparisons carry it: mandipropamid crystal vs predicted, and fludioxonil (0.71 A seed spread) vs benoxacor (3.27 A).</t>
         </is>
       </c>
       <c r="J4" s="9" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>ACTIVE (running)</t>
         </is>
       </c>
       <c r="K4" s="7" t="inlineStr">
@@ -1205,59 +1289,59 @@
       </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
-          <t>139-142, 161-164; jobs 27978561, 27981866</t>
+          <t>179, 180; job 27992285</t>
         </is>
       </c>
     </row>
     <row r="5" ht="108" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Decoded true-negative label set (Park Fig 5)</t>
+          <t>RFdiffusion3 motif scaffolding</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Design - benchmark</t>
+          <t>Scaffold - design</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Programmatic decoding of a published figure: each substitution cell is a 2x2 block, one sub-cell per compound, positions anchored to the label glyphs.</t>
+          <t>Diffusion scaffolding around the four HAB1-interface segments held as a fixed motif, with wide linker ranges so scaffold length and therefore envelope can vary.</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Supplied the first true negatives in the project. Every metric before this was recall-only because the ground truth was positive-unlabeled.</t>
+          <t>Revisits 7's rejection. That objection was about the two-state switch, NOT about cavity generation, and 85 removed its discriminating power -- no design of any kind can now be shown to cycle.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>475 variants x 15 agrochemicals in the K59R background</t>
+          <t>PYR1 chain A, residues 1-181; motif A60-63/A84-89/A115-117/A148-166</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Sep 1</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>7,045 TRUE NEGATIVES against 80 positives. 5,833 of them follow from the caption and the compound list alone; only 1,292 cells needed decoding. Quadrant-to-compound mapping verified with zero cross-contamination. Also corrected the benchmark itself: K59R was FORCED, not selected, and V81I is a benzothiadiazole hit rather than a mandipropamid one.</t>
+          <t>QUEUED behind the pose-check MD. Residue numbering asserted before submission: all 19 interface residues present with expected identities, gaps only at 69-70 which fall in a rebuilt linker.</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Responsiveness is not affinity, and cross-reactivity is a separate axis this set does not resolve. 8 of the 25 residues are absent from the figure and are negative by omission.</t>
+          <t>Fixing the C-lobe span freezes F159/V163/V164, which are pocket wall, so depth gain is one-sided. Inherent to preserving the interface. A prior RF3 attempt in the sibling project failed on a config API mismatch.</t>
         </is>
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>Score a variant only against the ligand whose pose was modelled. Comparing a benoxacor responder against the mandipropamid pose asks about a molecule twice the size of the one it binds.</t>
+          <t>Scored on ENVELOPE not cavity volume (106). Batch 2 is specified with Jannis's minimal loop anchors: 54 residues covering all 19 interface positions, against 139 for the literal extend-to-structure reading.</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>ACTIVE (running)</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1267,64 +1351,64 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>GPU short_gpu</t>
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>149, 156, 160, 166</t>
+          <t>183; job 27994380</t>
         </is>
       </c>
     </row>
     <row r="6" ht="108" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Clash-relief scope test (four ligands, own poses)</t>
+          <t>Thermodynamic integration (TI)</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Design - scoring</t>
+          <t>Affinity - energetics</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Park's 475 scored against each compound's own pose, so that pose confidence and ligand chemistry vary independently.</t>
+          <t>Alchemical free-energy difference along a lambda path with softcore; two legs give a selectivity ddG.</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Asked what the AUC 0.868 mandipropamid result actually measures.</t>
+          <t>Asked whether TI can rank PYR1 point mutations well enough to choose between them.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>mandipropamid (crystal) + 3 agrochemicals (predicted)</t>
+          <t>PYR1 + ABA / mandipropamid; 85-88, 90-92</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Aug 22-24</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid AUC 0.868 (p &lt; 1e-4, 11 of 20 positives in the top 25); fludioxonil 0.550, benzothiadiazole 0.528, benoxacor 0.469, all at chance with ZERO positives in the top 25. The cause is not the pose: mandipropamid strains the unmutated pocket by +1501 REU while the three agrochemicals, at 13-18 heavy atoms against its 30, strain it by -6.5 to +36.4. They already fit, so there is no clash to relieve.</t>
+          <t>A working Amber TI pipeline with six setup traps documented. The pilot ran 72/72 and the quadruple 48/48. The crystal arm gives the right SIGN and NO CALL at +-2.34 kcal/mol against an effect of ~1.</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>The scope is narrower than 91 implied: it answers which mutation makes ROOM for a ligand too big for the pocket, and is silent on which mutation makes a pocket bind a ligand that already fits. Size does not predict strain -- WIN 55,212-2 is 32 heavy atoms and strains PYL2 by only +15.7.</t>
+          <t>The docked arm is structurally invalid -- the ligand collapses into deleted F108's volume, which breaks the whole dock-into-an-enlarged-pocket workflow. The pilot's own error bar was 20x too small until a regex double-counting frames was found.</t>
         </is>
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid is the only large, clashing, positively-labelled ligand in the corpus, so the comparison cannot be made by adding a ligand. Isolate the pose variable instead (167).</t>
-        </is>
-      </c>
-      <c r="J6" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>8.3 GPU-days per variant pair is the real cost, which is what moved the project off affinity prediction and onto library enrichment (47).</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>RETIRED</t>
         </is>
       </c>
       <c r="K6" s="7" t="inlineStr">
@@ -1334,64 +1418,64 @@
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab</t>
+          <t>GPU</t>
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr">
         <is>
-          <t>165, 166, 167</t>
+          <t>85-92; jobs 27725295 and predecessors</t>
         </is>
       </c>
     </row>
     <row r="7" ht="108" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Forcing rule for library positions</t>
+          <t>Umbrella sampling of the open/closed coordinate</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Design - library</t>
+          <t>Conformation - energetics</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Two-part statistic: P(position mutated | ligand class) and P(residue | mutated, class), used to force a position into a library menu.</t>
+          <t>62 windows along P88 CA - R116 CA with WHAM, forward and reverse seeded, holo and apo.</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Asked whether a shallow menu at a productive position beats a deep menu at an unproductive one.</t>
+          <t>The last route to the open/closed dG that unbiased MD cannot reach (62), and so to the switching cost of a designed pocket.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Tian sd03/sd07 coumarin and PFAS arms</t>
+          <t>S1/S2/S9/S10 factorial seeds; 1.24 us biased</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Aug 25-26</t>
+          <t>Aug 25-28</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>Forcing is a real lever at shallow positions, and V163W was callable in advance. On PFAS the headroom is POSITIONAL, not identity: 3,441x collapses to 192x once the &lt;=6 substitution depth cap is applied to both sides.</t>
+          <t>FAILS its own pre-registered test. Forward and reverse disagree by 3.22 kcal/mol holo and 2.74 apo against a half-split drift bar of 0.22 and 1.05, and the SIGN of the tilt flips between seedings (+4.61 vs -3.29). Calibration also fails on its own terms (ddG -1.90 where a pass needs positive).</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>P(top | mutated) was partly circular -- 1.00 by construction wherever the library offered a single option.</t>
+          <t>My own 70/127 repair destroyed the two-directional seeding, which 81b suspected and 85 confirmed. Separately, the seeds came from only 5 of the 11 finished factorial trajectories (see the extraction bug below).</t>
         </is>
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>The vocabulary is closed; the win is new positions. Confirmed independently on Beltran-45, where Tian's frequency prior saturates exactly at the 67 % vocabulary ceiling.</t>
-        </is>
-      </c>
-      <c r="J7" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>A 15x miss with a sign flip is protocol, not sampling length. Do not rerun. Switch cost is a Y2H question.</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>RETIRED</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1401,62 +1485,62 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>GPU short_gpu</t>
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>116-119, 128, 153</t>
+          <t>111-113, 127, 136, 138; jobs 27854551</t>
         </is>
       </c>
     </row>
     <row r="8" ht="108" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Cavity chamber decomposition (bottleneck radius)</t>
+          <t>Boltz-2 co-folding and affinity head</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Pocket - structure</t>
+          <t>Affinity - ML</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Decomposes an enclosed cavity into chambers by the MAXIMIN of clearance along paths between them - the largest sphere that can be walked from one to the other. Exact on the grid; makes no straight-pocket assumption.</t>
+          <t>Structure + binding prediction from sequence and SMILES; affinity_probability_binary and affinity_pred_value.</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Re-measured PYR1 and 19 relatives after the total-volume comparison was shown to be counting voids a ligand cannot reach.</t>
+          <t>Asked three separate questions: can it rank pocket VARIANTS, can it predict ligand TRACTABILITY, and can it supply poses for ligands with no crystal structure.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>PYR1 3QN1 frame + 10 large-cavity relatives</t>
+          <t>718 sensor structures; 362 property-matched tractability models; 50 pose predictions</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>Aug 28</t>
+          <t>Aug 27-31</t>
         </is>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>A QUARTER of PYR1's own published cavity volume is satellite, not chamber: 164 total but 119 main. Only 2PCS has a genuinely large single chamber (570/570, r_max 3.80); 2NS9 462/157, 6AWV 305/126 with satellites behind r = 1.43 necks, 3QRZ 212/73. The large totals are mostly fragmentation.</t>
+          <t>Variant ranking: NO (within-ligand rho -0.028, and the binder classifier calls 90 % of real sensors non-binders). Poses: it finds the right pocket every time and builds the CLOSED receptor (gate RMSD 1.15-1.80 A), with a single consistent pose for about a quarter of ligands (97 of 362 under 1.0 A).</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Only detects constrictions that SEPARATE chambers - a waist within one chamber is invisible to it, which is what Jannis saw in PyMOL for 4DSB. Volume split between chambers is nearest-seed Voronoi, approximate at boundaries; the bottleneck radii themselves are exact.</t>
+          <t>Two silent failures cost whole arrays: a single trailing NUL byte in the shared a3m, and a ONE-RESIDUE mismatch between the a3m query and the input sequence, which makes it abandon the MSA and fold single-sequence at pLDDT 49 instead of 96. Neither errors.</t>
         </is>
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Report chamber volume, never total enclosed volume, when comparing pockets across structures. Two earlier metrics of mine were withdrawn on the way here: a circular C-beta envelope, and a poly-Gly column that reported 0-3 A^3 when the component ceased to exist.</t>
-        </is>
-      </c>
-      <c r="J8" s="9" t="inlineStr">
+          <t>Assert the fold (median pLDDT &gt;= 80) and assert the a3m query equals the input sequence, before any downstream number is computed.</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1468,19 +1552,19 @@
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>GPU short_gpu</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
-          <t>143, 145, 150, 151, 152</t>
+          <t>139-142, 161-164; jobs 27978561, 27981866</t>
         </is>
       </c>
     </row>
     <row r="9" ht="108" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Library recall on Beltran-45 (held-out benchmark)</t>
+          <t>Decoded true-negative label set (Park Fig 5)</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1490,40 +1574,40 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Scores a LIBRARY, not a variant: a menu of positions x allowed residues, size prod(1+n_i); a sensor is captured when all its substitutions lie inside. Recall at fixed size, never precision.</t>
+          <t>Programmatic decoding of a published figure: each substitution cell is a 2x2 block, one sub-cell per compound, positions anchored to the label glyphs.</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>First genuinely held-out test in the project - 45 cannabinoid sensors nothing here was built on, using 20 design positions of which only 10 overlap Tian's.</t>
+          <t>Supplied the first true negatives in the project. Every metric before this was recall-only because the ground truth was positive-unlabeled.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Beltran 45 sensors; Tian sd03 as the frequency prior</t>
+          <t>475 variants x 15 agrochemicals in the K59R background</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Aug 28</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Tian's substitution frequency TRANSFERS: 64 % recall at a library of 1e5 against a random null of 15 % +- 13 % (p &lt; 0.001), 33 % at 1e3 against 4 %. But it saturates at exactly the vocabulary ceiling - Tian's whole 144-substitution vocabulary captures 30/45 = 67 % - so all remaining headroom is POSITIONAL. CBDA 0/3, THC 0/2 and 4F-MDMB 0/1 are unreachable however the 144 are re-ranked.</t>
+          <t>7,045 TRUE NEGATIVES against 80 positives. 5,833 of them follow from the caption and the compound list alone; only 1,292 cells needed decoding. Quadrant-to-compound mapping verified with zero cross-contamination. Also corrected the benchmark itself: K59R was FORCED, not selected, and V81I is a benzothiadiazole hit rather than a mandipropamid one.</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Beltran's sensors came from Beltran's libraries, so a position they never varied is invisible: absence is not evidence against a position.</t>
+          <t>Responsiveness is not affinity, and cross-reactivity is a separate axis this set does not resolve. 8 of the 25 residues are absent from the figure and are negative by omission.</t>
         </is>
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>The win is new POSITIONS, not re-ranking the known vocabulary. Any new library method must beat the frequency baseline, which is advantaged and hard to beat.</t>
-        </is>
-      </c>
-      <c r="J9" s="9" t="inlineStr">
+          <t>Score a variant only against the ligand whose pose was modelled. Comparing a benoxacor responder against the mandipropamid pose asks about a molecule twice the size of the one it binds.</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1540,14 +1624,14 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>149, 156, 160, 166</t>
         </is>
       </c>
     </row>
     <row r="10" ht="108" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Single-substitution ddG at Beltran's 20 positions</t>
+          <t>Clash-relief scope test (four ligands, own poses)</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -1557,40 +1641,40 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>All 380 singles by protein-only Cartesian FastRelax ddG with a paired same-shell wild-type control; 3 replicates, minimum taken.</t>
+          <t>Park's 475 scored against each compound's own pose, so that pose confidence and ligand chemistry vary independently.</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Asked the per-RESIDUE false-negative question: if ddG chose the library, which real substitutions would be discarded?</t>
+          <t>Asked what the AUC 0.868 mandipropamid result actually measures.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>PYR1 3QN1 frame; Beltran's 20 design positions</t>
+          <t>mandipropamid (crystal) + 3 agrochemicals (predicted)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Aug 28-31</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Replicate spread measured for the first time: median 0.00, 90th pct 0.21 REU, against a ~2.7 REU signal - the score is PRECISE, so imprecision is not the problem. Recall if ddG chose the library: 22 % at top-10 %, 42 % at top-25 %, and 52 % at top-50 % which is chance. AUC 0.606. ref2015 penalises SHRINK substitutions specifically (median +2.40 vs +0.54 grow) and real sensors are shrink-biased (median dV -16.3 vs -3.7), so it penalises the class it should favour.</t>
+          <t>Mandipropamid AUC 0.868 (p &lt; 1e-4, 11 of 20 positives in the top 25); fludioxonil 0.550, benzothiadiazole 0.528, benoxacor 0.469, all at chance with ZERO positives in the top 25. The cause is not the pose: mandipropamid strains the unmutated pocket by +1501 REU while the three agrochemicals, at 13-18 heavy atoms against its 30, strain it by -6.5 to +36.4. They already fit, so there is no clash to relieve.</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Y120G, the most widely used substitution in the whole set, ranks 356/380. A volume correction fitted label-free lifted AUC to 0.666 on this set but FAILED to transfer to mandipropamid and is withdrawn.</t>
+          <t>The scope is narrower than 91 implied: it answers which mutation makes ROOM for a ligand too big for the pocket, and is silent on which mutation makes a pocket bind a ligand that already fits. Size does not predict strain -- WIN 55,212-2 is 32 heavy atoms and strains PYL2 by only +15.7.</t>
         </is>
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>The filter is a clash detector suitable as a final viability screen on an already-narrow set, not as the thing that does the narrowing.</t>
-        </is>
-      </c>
-      <c r="J10" s="9" t="inlineStr">
+          <t>Mandipropamid is the only large, clashing, positively-labelled ligand in the corpus, so the comparison cannot be made by adding a ligand. Isolate the pose variable instead (167).</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1607,57 +1691,57 @@
       </c>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>154, 157, 158</t>
+          <t>165, 166, 167</t>
         </is>
       </c>
     </row>
     <row r="11" ht="108" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Closed-space enumeration (Park-475, DSM doubles)</t>
+          <t>Forcing rule for library positions</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Design - benchmark</t>
+          <t>Design - library</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Exhaustive scoring of a real published library in its own defined search space: Park's 475 site-saturation singles in the K59R backbone, and all 35,863 allowed doubles of Beltran's DSM library.</t>
+          <t>Two-part statistic: P(position mutated | ligand class) and P(residue | mutated, class), used to force a position into a library menu.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>The sharpest available retrospective test - the search space is closed and stated in the papers' methods, so ranks are interpretable.</t>
+          <t>Asked whether a shallow menu at a productive position beats a deep menu at an unproductive one.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>4WVO mandi pose in the PYR1 frame; 7MWN reverted to wild-type PYL2 with WI5</t>
+          <t>Tian sd03/sd07 coumarin and PFAS arms</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Aug 31</t>
+          <t>Aug 25-26</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>DSM doubles: the five round-1 WIN hits rank 1547, 4805, 6632, 8276, 17532 of 35,863; median 6632 vs a null median 17,935, permutation p = 0.047. Screen size to a first hit 1547 vs 7172 expected - a 4.6x narrowing, the first such number on a closed independently-defined library. Park-475: F108A ranks 2/475 but the whole top 12 is F108X at -1358 to -1484 REU, V81I 260 and F159L 146.</t>
+          <t>Forcing is a real lever at shallow positions, and V163W was callable in advance. On PFAS the headroom is POSITIONAL, not identity: 3,441x collapses to 192x once the &lt;=6 substitution depth cap is applied to both sides.</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>It finds A160 (2.63x enriched in the top 1 %) and is BLIND to F159 (1.03x, exactly chance) although all five hits pair them. The conditional test refutes the greedy hypothesis: V81I stays at 224/222/221 across K59R, +F108A and +F108A+F159L backgrounds, and the score prefers V81F and V81Y at ranks 7-8.</t>
+          <t>P(top | mutated) was partly circular -- 1.00 by construction wherever the library offered a single option.</t>
         </is>
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Jannis found the benchmark itself was wrong: the mandi library was built in the FORCED K59R backbone, so every earlier record of 'K59R is invisible to every method' was scoring a prediction nobody had to make.</t>
-        </is>
-      </c>
-      <c r="J11" s="9" t="inlineStr">
+          <t>The vocabulary is closed; the win is new positions. Confirmed independently on Beltran-45, where Tian's frequency prior saturates exactly at the 67 % vocabulary ceiling.</t>
+        </is>
+      </c>
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1669,19 +1753,19 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>156, 159, 160</t>
+          <t>116-119, 128, 153</t>
         </is>
       </c>
     </row>
     <row r="12" ht="108" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Cavity characterisation (lib_cavity)</t>
+          <t>Cavity chamber decomposition (bottleneck radius)</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -1691,40 +1775,40 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Grid-based cavity detection; volume from probe-accessible grid points, with residues assigned by cavity lining + line of sight rather than distance to ligand.</t>
+          <t>Decomposes an enclosed cavity into chambers by the MAXIMIN of clearance along paths between them - the largest sphere that can be walked from one to the other. Exact on the grid; makes no straight-pocket assumption.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Defined the pocket, measured expansion per variant, found the length limit and the lobe gatekeeper.</t>
+          <t>Re-measured PYR1 and 19 relatives after the total-volume comparison was shown to be counting voids a ligand cannot reach.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>ABA (A8S); 3QN1, 3K3K, +7 deposited PYR1 chains</t>
+          <t>PYR1 3QN1 frame + 10 large-cavity relatives</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Aug 6-10</t>
+          <t>Aug 28</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Two findings about DIFFERENT states, which must not be compressed into one sentence. In WILD TYPE the satellite lobe is a sealed void, not connected to the ABA cavity, in 7 of 7 deposited chains - and F108 is the wall that seals it. In the QUAD mutant (K59/F108/E94/R79 truncated) the two lobes have fully merged into one continuous chamber with NO constriction: cross-sectional radius 4.0-6.3 A along the main span, and the apparent 'neck' at 5.02 A is the shallow minimum of a broad plateau. So the remaining limit is ligand LENGTH, not a bottleneck - the only narrow region is the gate/latch tail (1.4-2.7 A).</t>
+          <t>A QUARTER of PYR1's own published cavity volume is satellite, not chamber: 164 total but 119 main. Only 2PCS has a genuinely large single chamber (570/570, r_max 3.80); 2NS9 462/157, 6AWV 305/126 with satellites behind r = 1.43 necks, 3QRZ 212/73. The large totals are mostly fragmentation.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Distance-to-ligand mislabelled E94 as second shell (it is first shell, 4.33 A).</t>
+          <t>Only detects constrictions that SEPARATE chambers - a waist within one chamber is invisible to it, which is what Jannis saw in PyMOL for 4DSB. Volume split between chambers is nearest-seed Voronoi, approximate at boundaries; the bottleneck radii themselves are exact.</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Define pocket residues by cavity lining and line of sight, not a distance cutoff. R79 is a cavity-rim residue.</t>
-        </is>
-      </c>
-      <c r="J12" s="9" t="inlineStr">
+          <t>Report chamber volume, never total enclosed volume, when comparing pockets across structures. Two earlier metrics of mine were withdrawn on the way here: a circular C-beta envelope, and a poly-Gly column that reported 0-3 A^3 when the component ceased to exist.</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1741,124 +1825,124 @@
       </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>00-04, lib_cavity.py</t>
+          <t>143, 145, 150, 151, 152</t>
         </is>
       </c>
     </row>
     <row r="13" ht="108" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Foldseek + CATH50 superfamily scan</t>
+          <t>Library recall on Beltran-45 (held-out benchmark)</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Pocket - structure</t>
+          <t>Design - benchmark</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Structural (not sequence) homology search over CATH50; hits re-fetched full-atom and their cavities measured.</t>
+          <t>Scores a LIBRARY, not a variant: a menu of positions x allowed residues, size prod(1+n_i); a sensor is captured when all its substitutions lie inside. Recall at fixed size, never precision.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Asked whether an SRPBCC relative already has a bigger pocket to borrow from.</t>
+          <t>First genuinely held-out test in the project - 45 cannabinoid sensors nothing here was built on, using 20 design positions of which only 10 overlap Tian's.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>266 structural hits; 147 full-atom cavities</t>
+          <t>Beltran 45 sensors; Tian sd03 as the frequency prior</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Aug 6-7</t>
+          <t>Aug 28</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Found CoxG (2pcsA00 / 8UDS): ~570-600 A^3 pockets vs PYR1's 174, evolved to extract C45 menaquinone from membranes.</t>
+          <t>Tian's substitution frequency TRANSFERS: 64 % recall at a library of 1e5 against a random null of 15 % +- 13 % (p &lt; 0.001), 33 % at 1e3 against 4 %. But it saturates at exactly the vocabulary ceiling - Tian's whole 144-substitution vocabulary captures 30/45 = 67 % - so all remaining headroom is POSITIONAL. CBDA 0/3, THC 0/2 and 4F-MDMB 0/1 are unreachable however the 144 are re-ranked.</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>CoxG's pocket is OPEN, which conflicts with PYR1's closed-state readout. Top-hit calls unstable to --max-seqs.</t>
+          <t>Beltran's sensors came from Beltran's libraries, so a position they never varied is invisible: absence is not evidence against a position.</t>
         </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>A large natural pocket in the same fold exists, but pocket size and allosteric readout are coupled - you cannot import one without the other.</t>
-        </is>
-      </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>OPTION</t>
+          <t>The win is new POSITIONS, not re-ranking the known vocabulary. Any new library method must beat the frequency baseline, which is advantaged and hard to beat.</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>03, 05, 08, 10</t>
+          <t>153</t>
         </is>
       </c>
     </row>
     <row r="14" ht="108" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Rosetta FastRelax cavity scan (Arm 1)</t>
+          <t>Single-substitution ddG at Beltran's 20 positions</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Pocket - energetics</t>
+          <t>Design - scoring</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>All-atom relax with ref2015, then dCavity vs WT across a designed variant panel.</t>
+          <t>All 380 singles by protein-only Cartesian FastRelax ddG with a paired same-shell wild-type control; 3 replicates, minimum taken.</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Ranked 41 pocket variants by how much cavity they open, x3 replicates.</t>
+          <t>Asked the per-RESIDUE false-negative question: if ddG chose the library, which real substitutions would be discarded?</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>ABA; 3QN1 closed, 3K3K open</t>
+          <t>PYR1 3QN1 frame; Beltran's 20 design positions</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Aug 6-7</t>
+          <t>Aug 28-31</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>Worked as intended: true between-variant sd 46.9 A^3, F = 139. Produced the variant portfolio.</t>
+          <t>Replicate spread measured for the first time: median 0.00, 90th pct 0.21 REU, against a ~2.7 REU signal - the score is PRECISE, so imprecision is not the problem. Recall if ddG chose the library: 22 % at top-10 %, 42 % at top-25 %, and 52 % at top-50 % which is chance. AUC 0.606. ref2015 penalises SHRINK substitutions specifically (median +2.40 vs +0.54 grow) and real sensors are shrink-biased (median dV -16.3 vs -3.7), so it penalises the class it should favour.</t>
         </is>
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Expansion does NOT predict switch cost (r = 0.03), so dCavity alone cannot rank designs.</t>
+          <t>Y120G, the most widely used substitution in the whole set, ranks 356/380. A volume correction fitted label-free lifted AUC to 0.666 on this set but FAILED to transfer to mandipropamid and is withdrawn.</t>
         </is>
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Cavity opening is measurable and reproducible, but it is a means to a portfolio, not a selection criterion.</t>
-        </is>
-      </c>
-      <c r="J14" s="9" t="inlineStr">
+          <t>The filter is a clash detector suitable as a final viability screen on an already-narrow set, not as the thing that does the narrowing.</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -1875,64 +1959,64 @@
       </c>
       <c r="M14" s="7" t="inlineStr">
         <is>
-          <t>09, 20; job 27260956</t>
+          <t>154, 157, 158</t>
         </is>
       </c>
     </row>
     <row r="15" ht="108" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Rosetta open-vs-closed ddG (Arm 2 / 2b)</t>
+          <t>Closed-space enumeration (Park-475, DSM doubles)</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Pocket - energetics</t>
+          <t>Design - benchmark</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Relax each variant in open and closed states; the ddG between them proxies the energetic cost of switching.</t>
+          <t>Exhaustive scoring of a real published library in its own defined search space: Park's 475 site-saturation singles in the K59R backbone, and all 35,863 allowed doubles of Beltran's DSM library.</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Tried to score whether an enlarged pocket still prefers the closed, HAB1-competent state.</t>
+          <t>The sharpest available retrospective test - the search space is closed and stated in the papers' methods, so ranks are interpretable.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>ABA; 3QN1 vs 3K3K; 41 variants at nstruct 3, 20, 12</t>
+          <t>4WVO mandi pose in the PYR1 frame; 7MWN reverted to wild-type PYL2 with WI5</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Aug 7-10</t>
+          <t>Aug 31</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Arm 2b reached F = 9.0 with a true spread of 1.79 REU.</t>
+          <t>DSM doubles: the five round-1 WIN hits rank 1547, 4805, 6632, 8276, 17532 of 35,863; median 6632 vs a null median 17,935, permutation p = 0.047. Screen size to a first hit 1547 vs 7172 expected - a 4.6x narrowing, the first such number on a closed independently-defined library. Park-475: F108A ranks 2/475 but the whole top 12 is F108X at -1358 to -1484 REU, V81I 260 and F159L 146.</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Arm 2 v1 was declared statistically blind - wrongly. The readout is INVARIANT, not blind: true spread 0.43-0.50 REU against a -67 REU interface.</t>
+          <t>It finds A160 (2.63x enriched in the top 1 %) and is BLIND to F159 (1.03x, exactly chance) although all five hits pair them. The conditional test refutes the greedy hypothesis: V81I stays at 224/222/221 across K59R, +F108A and +F108A+F159L backgrounds, and the score prefers V81F and V81Y at ranks 7-8.</t>
         </is>
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>A null is only a null if the assay can discriminate. Judge effects in physical units, not significance.</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>OPTION</t>
+          <t>Jannis found the benchmark itself was wrong: the mandi library was built in the FORCED K59R backbone, so every earlier record of 'K59R is invisible to every method' was scoring a prediction nobody had to make.</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -1942,57 +2026,57 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>22, 26, 32, 33; jobs 27275686, 27286483/4</t>
+          <t>156, 159, 160</t>
         </is>
       </c>
     </row>
     <row r="16" ht="108" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Corrected discrimination statistic</t>
+          <t>Cavity characterisation (lib_cavity)</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Pocket - statistics</t>
+          <t>Pocket - structure</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>F = s2_between / (s2_within / n), where s2 is the VARIANCE (standard deviation squared). The denominator s2_within/n is the squared standard error of the mean, so dividing the within-group variance by n IS the sqrt(n) correction written in variance units - the two are the same equation, not two.</t>
+          <t>Grid-based cavity detection; volume from probe-accessible grid points, with residues assigned by cavity lining + line of sight rather than distance to ligand.</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>Re-derived every arm's discrimination after finding the original statistic wrong.</t>
+          <t>Defined the pocket, measured expansion per variant, found the length limit and the lobe gatekeeper.</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>Re-analysis of existing Rosetta output; no new structures.</t>
+          <t>ABA (A8S); 3QN1, 3K3K, +7 deposited PYR1 chains</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Aug 10</t>
+          <t>Aug 6-10</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Flipped Arm 2b from 'blind' to F = 9.0, correcting a central project claim.</t>
+          <t>Two findings about DIFFERENT states, which must not be compressed into one sentence. In WILD TYPE the satellite lobe is a sealed void, not connected to the ABA cavity, in 7 of 7 deposited chains - and F108 is the wall that seals it. In the QUAD mutant (K59/F108/E94/R79 truncated) the two lobes have fully merged into one continuous chamber with NO constriction: cross-sectional radius 4.0-6.3 A along the main span, and the apparent 'neck' at 5.02 A is the shallow minimum of a broad plateau. So the remaining limit is ligand LENGTH, not a bottleneck - the only narrow region is the gate/latch tail (1.4-2.7 A).</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>The original statistic used s_within itself as the yardstick - it compared between-group spread to the scatter of a SINGLE replicate rather than to the scatter of the replicate MEAN, which is sqrt(n) times smaller. The error had already propagated into several conclusions before it was found.</t>
+          <t>Distance-to-ligand mislabelled E94 as second shell (it is first shell, 4.33 A).</t>
         </is>
       </c>
       <c r="I16" s="7" t="inlineStr">
         <is>
-          <t>Compare between-group spread against the SEM, not the replicate sd. Run the variance decomposition BEFORE concluding 'no effect'.</t>
-        </is>
-      </c>
-      <c r="J16" s="9" t="inlineStr">
+          <t>Define pocket residues by cavity lining and line of sight, not a distance cutoff. R79 is a cavity-rim residue.</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2009,14 +2093,14 @@
       </c>
       <c r="M16" s="7" t="inlineStr">
         <is>
-          <t>35_variance_decomposition.py</t>
+          <t>00-04, lib_cavity.py</t>
         </is>
       </c>
     </row>
     <row r="17" ht="108" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Arm 3 homolog cavity survey</t>
+          <t>Foldseek + CATH50 superfamily scan</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -2026,17 +2110,17 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Full-atom cavity measurement across foldseek homologs.</t>
+          <t>Structural (not sequence) homology search over CATH50; hits re-fetched full-atom and their cavities measured.</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Asked how PYR1's pocket compares to its structural family.</t>
+          <t>Asked whether an SRPBCC relative already has a bigger pocket to borrow from.</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>147 full-atom homolog structures</t>
+          <t>266 structural hits; 147 full-atom cavities</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -2046,20 +2130,20 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Placed PYR1's 174 A^3 pocket in family context; supported the CoxG lead.</t>
+          <t>Found CoxG (2pcsA00 / 8UDS): ~570-600 A^3 pockets vs PYR1's 174, evolved to extract C45 menaquinone from membranes.</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>First pass returned 0.0 A^3 for every cavity - foldseek stores Ca only, so convert2pdb emitted backbone traces. Silent and plausible-looking.</t>
+          <t>CoxG's pocket is OPEN, which conflicts with PYR1's closed-state readout. Top-hit calls unstable to --max-seqs.</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Validate a downloaded structure with the consuming tool before trusting a derived number. A zero can be a parsing artefact.</t>
-        </is>
-      </c>
-      <c r="J17" s="10" t="inlineStr">
+          <t>A large natural pocket in the same fold exists, but pocket size and allosteric readout are coupled - you cannot import one without the other.</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
         <is>
           <t>OPTION</t>
         </is>
@@ -2076,124 +2160,124 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>08, 10</t>
+          <t>03, 05, 08, 10</t>
         </is>
       </c>
     </row>
     <row r="18" ht="108" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>LigandMPNN</t>
+          <t>Rosetta FastRelax cavity scan (Arm 1)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Pocket - design</t>
+          <t>Pocket - energetics</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Graph neural network designing sequence conditioned on backbone AND explicit ligand atoms; outputs per-position amino-acid probabilities.</t>
+          <t>All-atom relax with ref2015, then dCavity vs WT across a designed variant panel.</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>Stage-1 retrospective test: can it recover the 4 known mandipropamid mutations from WT plus a perfectly placed ligand?</t>
+          <t>Ranked 41 pocket variants by how much cavity they open, x3 replicates.</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>Structures: WT PYR1 with mandipropamid (ligand 3UZ, from 4WVO) vs ABA (ligand A8S, from 3QN1) as the ligand-swap null.</t>
+          <t>ABA; 3QN1 closed, 3K3K open</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Aug 12</t>
+          <t>Aug 6-7</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>Recovered F108A (+0.111) and F159L (+0.071) with zero mass in the ABA arm - genuinely ligand-conditional.</t>
+          <t>Worked as intended: true between-variant sd 46.9 A^3, F = 139. Produced the variant portfolio.</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Missed K59R and V81I. V81I INVERTED (-0.841): ABA prefers Ile at 81 with p=0.996 in the arm whose answer is no mutations. Recovers only severe-clash positions, which a trivial clash baseline already gives free.</t>
+          <t>Expansion does NOT predict switch cost (r = 0.03), so dCavity alone cannot rank designs.</t>
         </is>
       </c>
       <c r="I18" s="7" t="inlineStr">
         <is>
-          <t>Sequence recovery is the wrong metric - a ligand-blind oracle reaches 79.1% on the same labels. Score probability MASS against a ligand-swap null, never recall-at-N.</t>
-        </is>
-      </c>
-      <c r="J18" s="10" t="inlineStr">
-        <is>
-          <t>OPTION</t>
+          <t>Cavity opening is measurable and reproducible, but it is a means to a portfolio, not a selection criterion.</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L18" s="7" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>CPU cutlerlab</t>
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr">
         <is>
-          <t>43, 46; job 27412775</t>
+          <t>09, 20; job 27260956</t>
         </is>
       </c>
     </row>
     <row r="19" ht="108" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Rosetta FastDesign</t>
+          <t>Rosetta open-vs-closed ddG (Arm 2 / 2b)</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Pocket - design</t>
+          <t>Pocket - energetics</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Monte Carlo sequence design with ref2015: repack and minimise while allowing identity changes at chosen positions.</t>
+          <t>Relax each variant in open and closed states; the ddG between them proxies the energetic cost of switching.</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>The physics arm of the same stage-1 test, chosen because it fails differently from a learned model.</t>
+          <t>Tried to score whether an enlarged pocket still prefers the closed, HAB1-competent state.</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid vs ABA, 15 designable positions</t>
+          <t>ABA; 3QN1 vs 3K3K; 41 variants at nstruct 3, 20, 12</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Aug 13</t>
+          <t>Aug 7-10</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Recovered F108A at frequency 1.000 vs 0.000 in the null - the cleanest single recovery of the stage.</t>
+          <t>Arm 2b reached F = 9.0 with a true spread of 1.79 REU.</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>F159L: right position, wrong identity (picks D/E). V81I inverted (-0.980). The NULL ARM FAILED ITS OWN CONTROL: with the cognate ligand it kept WT at 29% and K59 in 0% of trajectories.</t>
+          <t>Arm 2 v1 was declared statistically blind - wrongly. The readout is INVARIANT, not blind: true spread 0.43-0.50 REU against a -67 REU interface.</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>If the null also mutates a position, 'no signal' is inseparable from 'the protocol cannot hold a native contact'. K59R and V81I were uninterpretable, not negative.</t>
-        </is>
-      </c>
-      <c r="J19" s="10" t="inlineStr">
+          <t>A null is only a null if the assay can discriminate. Judge effects in physical units, not significance.</t>
+        </is>
+      </c>
+      <c r="J19" s="11" t="inlineStr">
         <is>
           <t>OPTION</t>
         </is>
@@ -2210,59 +2294,59 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>50, 51; job 27421344</t>
+          <t>22, 26, 32, 33; jobs 27275686, 27286483/4</t>
         </is>
       </c>
     </row>
     <row r="20" ht="108" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Favour-native weight sweep</t>
+          <t>Corrected discrimination statistic</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Pocket - calibration</t>
+          <t>Pocket - statistics</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Adds a bonus for retaining wild-type identity; swept 0.25/0.5/1.0/1.5 on the NULL arm only, criterion fixed before submission.</t>
+          <t>F = s2_between / (s2_within / n), where s2 is the VARIANCE (standard deviation squared). The denominator s2_within/n is the squared standard error of the mean, so dividing the within-group variance by n IS the sqrt(n) correction written in variance units - the two are the same equation, not two.</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Attempt to repair FastDesign's WT-retention failure.</t>
+          <t>Re-derived every arm's discrimination after finding the original statistic wrong.</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>ABA null arm</t>
+          <t>Re-analysis of existing Rosetta output; no new structures.</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Aug 13</t>
+          <t>Aug 10</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>WT recovery climbed 29 -&gt; 45 -&gt; 59 -&gt; 65 -&gt; 85%.</t>
+          <t>Flipped Arm 2b from 'blind' to F = 9.0, correcting a central project claim.</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>K59 stayed at 0% AT EVERY WEIGHT, including 1.5 where the packer is nearly frozen (3 distinct sequences in 10). No weight passed.</t>
+          <t>The original statistic used s_within itself as the yardstick - it compared between-group spread to the scatter of a SINGLE replicate rather than to the scatter of the replicate MEAN, which is sqrt(n) times smaller. The error had already propagated into several conclusions before it was found.</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>The calibration failing IS the answer, not a setback. Do not widen a sweep until a control agrees - that is tuning until it says what you want.</t>
+          <t>Compare between-group spread against the SEM, not the replicate sd. Run the variance decomposition BEFORE concluding 'no effect'.</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
         <is>
-          <t>RETIRED</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K20" s="7" t="inlineStr">
@@ -2272,69 +2356,69 @@
       </c>
       <c r="L20" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
-          <t>53, 54; job 27438220</t>
+          <t>35_variance_decomposition.py</t>
         </is>
       </c>
     </row>
     <row r="21" ht="108" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Per-residue energy decomposition</t>
+          <t>Arm 3 homolog cavity survey</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Pocket - diagnosis</t>
+          <t>Pocket - structure</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Breaks ref2015's total into per-term, per-residue contributions at one position.</t>
+          <t>Full-atom cavity measurement across foldseek homologs.</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Asked WHY K59 could not be retained.</t>
+          <t>Asked how PYR1's pocket compares to its structural family.</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>ABA anion + K59 in 3QN1</t>
+          <t>147 full-atom homolog structures</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Aug 13</t>
+          <t>Aug 6-7</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>THE KEY DIAGNOSIS. ref2015 correctly sees the salt bridge (Lys best fa_elec by 1.9 REU, only candidate earning hbond_sc) then pays +10.118 REU of Lazaridis-Karplus desolvation to bury the ammonium. Ile beats Lys by 4.211 REU; Arg is 2.274 WORSE than Lys.</t>
+          <t>Placed PYR1's 174 A^3 pocket in family context; supported the CoxG lead.</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Ruled out pose (K59 NZ 2.85 A from carboxylate) and ionisation (params sum -0.970 over 38 atoms) first, costing extra runs.</t>
+          <t>First pass returned 0.0 A^3 for every cavity - foldseek stores Ca only, so convert2pdb emitted backbone traces. Silent and plausible-looking.</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>Diagnose the mechanism before proposing a fix. This one number explained three downstream failures and told us exactly which stage to replace.</t>
-        </is>
-      </c>
-      <c r="J21" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Validate a downloaded structure with the consuming tool before trusting a derived number. A zero can be a parsing artefact.</t>
+        </is>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
+        <is>
+          <t>OPTION</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>later</t>
         </is>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -2344,14 +2428,14 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>55, 55b; job 27438909</t>
+          <t>08, 10</t>
         </is>
       </c>
     </row>
     <row r="22" ht="108" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Coupled moves (Kortemme)</t>
+          <t>LigandMPNN</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -2361,40 +2445,40 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Monte Carlo coupling sequence, side-chain, BACKBONE and ligand-pose moves - the published fix for fixed-backbone specificity design (5.75x on its own benchmark, 16/17 cases).</t>
+          <t>Graph neural network designing sequence conditioned on backbone AND explicit ligand atoms; outputs per-position amino-acid probabilities.</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>Re-ran stage 1 changing ONLY the sampler: same positions, same arms, same scoring rule.</t>
+          <t>Stage-1 retrospective test: can it recover the 4 known mandipropamid mutations from WT plus a perfectly placed ligand?</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid vs ABA; 50 trajectories/arm x 1000 trials, ligand_mode on</t>
+          <t>Structures: WT PYR1 with mandipropamid (ligand 3UZ, from 4WVO) vs ABA (ligand A8S, from 3QN1) as the ligand-swap null.</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Aug 19</t>
+          <t>Aug 12</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>F108A recovered cleanly (+0.74 against a 0.00 null). WT retention improved 29% -&gt; 42%.</t>
+          <t>Recovered F108A (+0.111) and F159L (+0.071) with zero mass in the ABA arm - genuinely ligand-conditional.</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>K59R still missed. Decisively: in the ABA arm - cognate ligand, K59 unambiguously correct - K59 was retained in 0% of 50 trajectories, identical to fixed backbone.</t>
+          <t>Missed K59R and V81I. V81I INVERTED (-0.841): ABA prefers Ile at 81 with p=0.996 in the arm whose answer is no mutations. Recovers only severe-clash positions, which a trivial clash baseline already gives free.</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>SAMPLING IS NOT THE LIMIT at the design stage. Lysine is in every rotamer library and IncludeCurrent was on. Confirms the scoring diagnosis with a second independent sampler.</t>
-        </is>
-      </c>
-      <c r="J22" s="10" t="inlineStr">
+          <t>Sequence recovery is the wrong metric - a ligand-blind oracle reaches 79.1% on the same labels. Score probability MASS against a ligand-swap null, never recall-at-N.</t>
+        </is>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t>OPTION</t>
         </is>
@@ -2406,131 +2490,131 @@
       </c>
       <c r="L22" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab, 100 tasks</t>
+          <t>GPU</t>
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>74, 74b; job 27560390</t>
+          <t>43, 46; job 27412775</t>
         </is>
       </c>
     </row>
     <row r="23" ht="108" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Per-position steric admissibility</t>
+          <t>Rosetta FastDesign</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Pocket - geometry</t>
+          <t>Pocket - design</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>For each position x each of 20 residues, place every library rotamer and ask whether ANY is clash-free against ligand and environment. Hard yes/no on Bondi radii, no score function.</t>
+          <t>Monte Carlo sequence design with ref2015: repack and minimise while allowing identity changes at chosen positions.</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Headroom check: does pure geometry narrow the residue choice per position?</t>
+          <t>The physics arm of the same stage-1 test, chosen because it fails differently from a learned model.</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>ABA vs mandipropamid, 26 pocket positions, WT backbone</t>
+          <t>Mandipropamid vs ABA, 15 designable positions</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Aug 18</t>
+          <t>Aug 13</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Clean negative in an afternoon: mean 14.7/20 admissible, ABA-mandi Jaccard 0.84.</t>
+          <t>Recovered F108A at frequency 1.000 vs 0.000 in the null - the cleanest single recovery of the stage.</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>DOES NOT CLEAR. Too permissive (9x narrowing where Tian's focused library is 50x smaller) and largely ligand-blind. All four ground-truth substitutions are admissible for BOTH ligands - recalled without being ligand-conditional.</t>
+          <t>F159L: right position, wrong identity (picks D/E). V81I inverted (-0.980). The NULL ARM FAILED ITS OWN CONTROL: with the cognate ligand it kept WT at 29% and K59 in 0% of trajectories.</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>YES, IT EXCLUDED REAL SENSOR MUTATIONS - but read the scope carefully. Against mandipropamid's OWN ground truth it excluded nothing: all four of K59R/V81I/F108A/F159L were admissible (the problem there was that they were admissible for ABA too). Against Beltran's cannabinoid sensors it wrongly excluded six real substitutions - 7% of in-pocket occurrences - and NONE of them come from a WIN sensor: V83W (JWH-007 x2, JWH-167), V83F (JWH-167), V164W (CBDA x2), V164H (JWH-015), A89V (JWH-193), E141F (CP 47,497). All NINE WIN sensors passed, and that is informative rather than lucky: every WIN mutation is F159-&gt;A/G/S/T (a shrink, always admissible), A160-&gt;I/L/V (a modest grow at a small residue), K59Q, or a surface position - exactly the substitution types a per-position filter can handle. The failures concentrate in the bulky aromatic GROWS (Trp, Phe, His at V83/V164) that need a partner shrink first. Caveat: all of these were scored in the ABA/mandipropamid pocket, not a cannabinoid-bound one, so it is not a clean test of them. Every miss was a GROW mutation, and real sensors are compensating shrink/grow PAIRS (F159A+A160I; Y120G+A160G in 27 and 23 of Beltran's 45 sensors) that a per-position filter structurally cannot see.</t>
-        </is>
-      </c>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>RETIRED</t>
+          <t>If the null also mutates a position, 'no signal' is inseparable from 'the protocol cannot hold a native contact'. K59R and V81I were uninterpretable, not negative.</t>
+        </is>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
+        <is>
+          <t>OPTION</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>later</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>CPU cutlerlab</t>
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>71_admissibility.py</t>
+          <t>50, 51; job 27421344</t>
         </is>
       </c>
     </row>
     <row r="24" ht="108" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Pairwise enumeration</t>
+          <t>Favour-native weight sweep</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Pocket - geometry</t>
+          <t>Pocket - calibration</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Enumerates mutation PAIRS against a jointly re-scored pocket. Objective = summed ligand-protein vdW overlap (additive, hence a cheap precompute) subject to not losing packing.</t>
+          <t>Adds a bonus for retaining wild-type identity; swept 0.25/0.5/1.0/1.5 on the NULL arm only, criterion fixed before submission.</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>The version of the combinatorial idea the data supports, after per-position menus failed.</t>
+          <t>Attempt to repair FastDesign's WT-retention failure.</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid (clashes in WT: 2.78 A, 7/29 atoms) vs ABA (fits: 0.22 A, 0/19) - a built-in negative control</t>
+          <t>ABA null arm</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Aug 18</t>
+          <t>Aug 13</t>
         </is>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>Best steric result so far: F108A rank 5, F159L rank 75, V81I rank 150 of 13,457 - 3 of 4 in the top 150, a 90x narrowing. Shrink/grow enriched to 62% of the top 200 vs 42% for ABA.</t>
+          <t>WT recovery climbed 29 -&gt; 45 -&gt; 59 -&gt; 65 -&gt; 85%.</t>
         </is>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>K59R at rank 3907 - blind BY CATEGORY, since K59 does not clash at all. Picks the right POSITIONS (81+108) with the wrong identity at 81.</t>
+          <t>K59 stayed at 0% AT EVERY WEIGHT, including 1.5 where the packer is nearly frozen (3 distinct sequences in 10). No weight passed.</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>An ADDITIVE objective cannot show synergy. Counting contacts within a flat 4.5 A rewards clashes (83W+163Y topped the Pareto front with relief -71.7 A).</t>
-        </is>
-      </c>
-      <c r="J24" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>The calibration failing IS the answer, not a setback. Do not widen a sweep until a control agrees - that is tuning until it says what you want.</t>
+        </is>
+      </c>
+      <c r="J24" s="10" t="inlineStr">
+        <is>
+          <t>RETIRED</t>
         </is>
       </c>
       <c r="K24" s="7" t="inlineStr">
@@ -2540,106 +2624,106 @@
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>CPU cutlerlab</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
-          <t>72_pairwise.py</t>
+          <t>53, 54; job 27438220</t>
         </is>
       </c>
     </row>
     <row r="25" ht="108" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Electrostatic / H-bond complementarity</t>
+          <t>Per-residue energy decomposition</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Pocket - geometry</t>
+          <t>Pocket - diagnosis</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Counts geometrically valid donor-acceptor pairs to the ligand plus a screened-Coulomb term. Deliberately models NO desolvation.</t>
+          <t>Breaks ref2015's total into per-term, per-residue contributions at one position.</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>The stage pairwise enumeration specified: score the non-clashing positions electrostatics can reach.</t>
+          <t>Asked WHY K59 could not be retained.</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>ABA (anion, -0.97) vs mandipropamid (neutral, +0.10)</t>
+          <t>ABA anion + K59 in 3QN1</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Aug 18</t>
+          <t>Aug 13</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Gets K59 right for ABA - Lys rank 1 via a bidentate salt bridge (NZ-O4 2.83 A, NZ-O3 3.31 A) where stage 1 kept it 0% of the time. The ref2015 pathology is genuinely absent.</t>
+          <t>THE KEY DIAGNOSIS. ref2015 correctly sees the salt bridge (Lys best fa_elec by 1.9 REU, only candidate earning hbond_sc) then pays +10.118 REU of Lazaridis-Karplus desolvation to bury the ammonium. Ile beats Lys by 4.211 REU; Arg is 2.274 WORSE than Lys.</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Missed K59R. Fails its own controls in the PREDICTED direction: WT top choice at only 4% of positions, Lys/Arg picked at 59% against an anionic ligand - with no desolvation, everything wants to be charged.</t>
+          <t>Ruled out pose (K59 NZ 2.85 A from carboxylate) and ionisation (params sum -0.970 over 38 atoms) first, costing extra runs.</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>Not usable as a ranker; usable as a FILTER over supplied conformations. Its own miss was sampling: the crystal Arg59 (chi3 ~100 deg, non-rotameric) scores 2 H-bonds under its own criteria but is never proposed.</t>
-        </is>
-      </c>
-      <c r="J25" s="10" t="inlineStr">
-        <is>
-          <t>OPTION</t>
+          <t>Diagnose the mechanism before proposing a fix. This one number explained three downstream failures and told us exactly which stage to replace.</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>later</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>CPU cutlerlab</t>
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>73_electrostatic.py</t>
+          <t>55, 55b; job 27438909</t>
         </is>
       </c>
     </row>
     <row r="26" ht="108" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>Shared steric rule (lib_sterics)</t>
+          <t>Coupled moves (Kortemme)</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>Pocket - geometry</t>
+          <t>Pocket - design</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>One clash rule for all geometric screens: exempts donor-acceptor pairs down to 2.5 A, keeps acceptor-acceptor and donor-donor as clashes, includes a real hydrogen radius.</t>
+          <t>Monte Carlo coupling sequence, side-chain, BACKBONE and ligand-pose moves - the published fix for fixed-backbone specificity design (5.75x on its own benchmark, 16/17 cases).</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Fixed hydrogen bonds being scored as steric clashes across scripts 71/72/73.</t>
+          <t>Re-ran stage 1 changing ONLY the sampler: same positions, same arms, same scoring rule.</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>All pocket screens</t>
+          <t>Mandipropamid vs ABA; 50 trajectories/arm x 1000 trials, ligand_mode on</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -2649,87 +2733,87 @@
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>Unit-tested three ways. R79's crystal side chain goes from 0.306 A 'overlap' to 0.000. WT-ok at hard-sphere tolerance improved 12 -&gt; 16 of 26.</t>
+          <t>F108A recovered cleanly (+0.74 against a 0.00 null). WT retention improved 29% -&gt; 42%.</t>
         </is>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Did NOT rescue the R79/V83/H115 control failures - I had claimed it would. Those are rotamer-basin failures and the earlier diagnosis was right.</t>
+          <t>K59R still missed. Decisively: in the ABA arm - cognate ligand, K59 unambiguously correct - K59 was retained in 0% of 50 trajectories, identical to fixed backbone.</t>
         </is>
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>A hard-sphere test scores every hydrogen bond as a ~0.4 A clash. The fix was invisible at the 0.5 A tolerance in use, which already absorbed it - a stability check, not a revision.</t>
-        </is>
-      </c>
-      <c r="J26" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>SAMPLING IS NOT THE LIMIT at the design stage. Lysine is in every rotamer library and IncludeCurrent was on. Confirms the scoring diagnosis with a second independent sampler.</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>OPTION</t>
         </is>
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>later</t>
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr">
         <is>
-          <t>CPU local</t>
+          <t>CPU cutlerlab, 100 tasks</t>
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
-          <t>lib_sterics.py</t>
+          <t>74, 74b; job 27560390</t>
         </is>
       </c>
     </row>
     <row r="27" ht="108" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>MM-GBSA rescoring</t>
+          <t>Per-position steric admissibility</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Pocket - energetics</t>
+          <t>Pocket - geometry</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Replaces ref2015's pairwise Lazaridis-Karplus solvation with generalised Born: dG_bind = G_complex - G_receptor - G_ligand, averaged over an MD ensemble. ff14SB + GAFF2/AM1-BCC, igb=8, 0.15 M salt. Rosetta builds structures and never scores them.</t>
+          <t>For each position x each of 20 residues, place every library rotamer and ask whether ANY is clash-free against ligand and environment. Hard yes/no on Bondi radii, no score function.</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Direct attack on the diagnosed cause of the K59 failure.</t>
+          <t>Headroom check: does pure geometry narrow the residue choice per position?</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Mandipropamid vs ABA; 7 variants x 2 arms x 100-frame ensembles</t>
+          <t>ABA vs mandipropamid, 26 pocket positions, WT backbone</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Aug 19</t>
+          <t>Aug 18</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>⚠ THE K59 FLIP IS RETRACTED (README 40). It was an artefact of an UNCONVERGED reference: the WT-ABA complex moves +7.75 kcal/mol between 50 and 250 ps and is still drifting. Recomputed at 250 ps the pre-registered test gives the OPPOSITE answer, selectivity -8.58 (PASS) -&gt; +1.31 (FAIL). Sign-based verdicts from this method are void at these lengths; rank-based ones survive but are marginal (p = 0.049) and bounded by a 1.05 kcal/mol per-variant drift, the size of the spacing being ranked. README 42-43 retire it: +-3.85 needs n=60/variant, about 1748 GPU-hours.</t>
+          <t>Clean negative in an afternoon: mean 14.7/20 admissible, ABA-mandi Jaccard 0.84.</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Ensembles only 50 ps (GBn2 runs ~380 steps/min here; pmemd no faster). The ligand-swap difference is dominated by DAMAGE TO THE ABA COMPLEX, not gain for mandipropamid. F108A comes out NULL because relaxation absorbs the clash it exists to relieve.</t>
+          <t>DOES NOT CLEAR. Too permissive (9x narrowing where Tian's focused library is 50x smaller) and largely ligand-blind. All four ground-truth substitutions are admissible for BOTH ligands - recalled without being ligand-conditional.</t>
         </is>
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>Changing the solvation model does what no sampler could - the desolvation diagnosis was right AND actionable. Also: my first error bars were fabricated (8 'independent' repacks came out byte-identical).</t>
-        </is>
-      </c>
-      <c r="J27" s="8" t="inlineStr">
+          <t>YES, IT EXCLUDED REAL SENSOR MUTATIONS - but read the scope carefully. Against mandipropamid's OWN ground truth it excluded nothing: all four of K59R/V81I/F108A/F159L were admissible (the problem there was that they were admissible for ABA too). Against Beltran's cannabinoid sensors it wrongly excluded six real substitutions - 7% of in-pocket occurrences - and NONE of them come from a WIN sensor: V83W (JWH-007 x2, JWH-167), V83F (JWH-167), V164W (CBDA x2), V164H (JWH-015), A89V (JWH-193), E141F (CP 47,497). All NINE WIN sensors passed, and that is informative rather than lucky: every WIN mutation is F159-&gt;A/G/S/T (a shrink, always admissible), A160-&gt;I/L/V (a modest grow at a small residue), K59Q, or a surface position - exactly the substitution types a per-position filter can handle. The failures concentrate in the bulky aromatic GROWS (Trp, Phe, His at V83/V164) that need a partner shrink first. Caveat: all of these were scored in the ABA/mandipropamid pocket, not a cannabinoid-bound one, so it is not a clean test of them. Every miss was a GROW mutation, and real sensors are compensating shrink/grow PAIRS (F159A+A160I; Y120G+A160G in 27 and 23 of Beltran's 45 sensors) that a per-position filter structurally cannot see.</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
         <is>
           <t>RETIRED</t>
         </is>
@@ -2741,62 +2825,62 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>CPU cutlerlab, 14 tasks</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>75, 75b-e; jobs 27561665, 27568930, 27569546</t>
+          <t>71_admissibility.py</t>
         </is>
       </c>
     </row>
     <row r="28" ht="108" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Coumarin focused-library benchmark</t>
+          <t>Pairwise enumeration</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>Pocket - benchmark</t>
+          <t>Pocket - geometry</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Extracts the exact per-position residue menus Tian et al. built for each focused library, then measures what a method must add over a ligand-blind baseline.</t>
+          <t>Enumerates mutation PAIRS against a jointly re-scored pocket. Objective = summed ligand-protein vdW overlap (additive, hence a cheap precompute) subject to not losing packing.</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Asked whether round-1 screening could have been skipped computationally.</t>
+          <t>The version of the combinatorial idea the data supports, after per-position menus failed.</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>LIBRARY DESIGNS, not structures: Tian sd04 per-position residue menus for the Coumarin, PFAS and TNTv1/v2 focused libraries, plus 692 characterised sensor clones (sequences).</t>
+          <t>Mandipropamid (clashes in WT: 2.78 A, 7/29 atoms) vs ABA (fits: 0.22 A, 0/19) - a built-in negative control</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Aug 14</t>
+          <t>Aug 18</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>Reframed the task. POSITIONS are near ligand-independent: Coumarin/PFAS/TNTv2 share 9 of their 11-14 positions, so naming the shared nine scores 82% recall with ZERO ligand information. SUBSTITUTIONS are ligand-specific: mean 3-way Jaccard 0.02.</t>
+          <t>Best steric result so far: F108A rank 5, F159L rank 75, V81I rank 150 of 13,457 - 3 of 4 in the top 150, a 90x narrowing. Shrink/grow enriched to 62% of the top 200 vs 42% for ABA.</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>I initially claimed the coumarin library design was missing from the supplement. It was not - a column header truncated at 20 characters.</t>
+          <t>K59R at rank 3907 - blind BY CATEGORY, since K59 does not clash at all. Picks the right POSITIONS (81+108) with the wrong identity at 81.</t>
         </is>
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>Predict MENUS, not positions. Focusing buys ~16 orders of magnitude (3.8e21 -&gt; 1.4e5).</t>
-        </is>
-      </c>
-      <c r="J28" s="9" t="inlineStr">
+          <t>An ADDITIVE objective cannot show synergy. Counting contacts within a flat 4.5 A rewards clashes (83W+163Y topped the Pareto front with relief -71.7 A).</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2813,64 +2897,64 @@
       </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
-          <t>62_coumarin_ground_truth.py</t>
+          <t>72_pairwise.py</t>
         </is>
       </c>
     </row>
     <row r="29" ht="108" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Beltran cannabinoid sensor table</t>
+          <t>Electrostatic / H-bond complementarity</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Pocket - benchmark</t>
+          <t>Pocket - geometry</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>45 experimentally validated sensors across 12 cannabinoids, with mutation sets and a graded dose-response (1e4 -&gt; 10 nM).</t>
+          <t>Counts geometrically valid donor-acceptor pairs to the ligand plus a screened-Coulomb term. Deliberately models NO desolvation.</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>A second, harder ground truth with an ORDER to recover, not just a set.</t>
+          <t>The stage pairwise enumeration specified: score the non-clashing positions electrostatics can reach.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Sensor SEQUENCE table (no solved structures): 45 PYR1 variants vs WIN 55,212-2, the JWH series, D9-THC, CBDA, CP 47,497. WIN 55,212-2 is an aminoalkylindole synthetic cannabinoid, so it belongs in this set despite the name looking unlike the others.</t>
+          <t>ABA (anion, -0.97) vs mandipropamid (neutral, +0.10)</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Aug 18-19</t>
+          <t>Aug 18</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Extracted in full. A160 mutated in 38/45, Y120 in 33/45, F159 in 24/45. Ligand-specific signal sits at K59 (Q/N/S/T/A/R), H115Q, V83, E141, V164, V81.</t>
+          <t>Gets K59 right for ABA - Lys rank 1 via a bidentate salt bridge (NZ-O4 2.83 A, NZ-O3 3.31 A) where stage 1 kept it 0% of the time. The ref2015 pathology is genuinely absent.</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Even more position-saturated than coumarin; substitutions reused within a chemical family (A160G 27x, Y120G 23x). Nine substitutions sit OUTSIDE the 5 A pocket - PYR1-WIN gets its last order of magnitude from E4G.</t>
+          <t>Missed K59R. Fails its own controls in the PREDICTED direction: WT top choice at only 4% of positions, Lys/Arg picked at 59% against an anionic ligand - with no desolvation, everything wants to be charged.</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>A graded sensitivity ladder is a far stronger benchmark than a hit list. K59Q/K59N are neutral, so they should be reachable where K59R was not - a free sanity check.</t>
-        </is>
-      </c>
-      <c r="J29" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Not usable as a ranker; usable as a FILTER over supplied conformations. Its own miss was sampling: the crystal Arg59 (chi3 ~100 deg, non-rotameric) scores 2 H-bonds under its own criteria but is never proposed.</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr">
+        <is>
+          <t>OPTION</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>later</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -2880,34 +2964,34 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>data/beltran/win_sensors.json</t>
+          <t>73_electrostatic.py</t>
         </is>
       </c>
     </row>
     <row r="30" ht="108" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Literature protocol review</t>
+          <t>Shared steric rule (lib_sterics)</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Pocket - benchmark</t>
+          <t>Pocket - geometry</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Read six papers from their Methods sections, not abstracts, to establish what the field does and what the honest baseline is.</t>
+          <t>One clash rule for all geometric screens: exempts donor-acceptor pairs down to 2.5 A, keeps acceptor-acceptor and donor-donor as clashes, includes a real hydrogen radius.</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Calibrated our results against published practice before investing further.</t>
+          <t>Fixed hydrogen bonds being scored as steric clashes across scripts 71/72/73.</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Six papers (PDFs + extracted Methods text): Leonard 2026, An 2024, Tian 2025, Park 2023, ACS Chem Biol 2024, Nat Biotech 2026.</t>
+          <t>All pocket screens</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -2917,20 +3001,20 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>Leonard's 'dock to sequence' MUTATES WT to a known weak-hit sequence before placing any pose - their method improves a known weak binder and cannot start from a ligand alone. An et al. picked cutoffs by MANUAL INSPECTION. RbsB precedent: 2M variants screened for 1.2-1.5x induction.</t>
+          <t>Unit-tested three ways. R79's crystal side chain goes from 0.306 A 'overlap' to 0.000. WT-ok at hard-sphere tolerance improved 12 -&gt; 16 of 26.</t>
         </is>
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Leonard hard-filters on an H-bond to the latch water, which mandipropamid misses by 5.07-5.19 A - their protocol would reject the correct pose.</t>
+          <t>Did NOT rescue the R79/V83/H115 control failures - I had claimed it would. Those are rotamer-basin failures and the earlier diagnosis was right.</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>The field's baseline is low, and our benchmark is strictly harder than Leonard's. The ACS Chem Biol paper independently confirmed R79 H-bonds F52's carbonyl at &gt;90% occupancy, explaining one of our control failures from the other direction.</t>
-        </is>
-      </c>
-      <c r="J30" s="9" t="inlineStr">
+          <t>A hard-sphere test scores every hydrogen bond as a ~0.4 A clash. The fix was invisible at the 0.5 A tolerance in use, which already absorbed it - a stability check, not a revision.</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -2942,64 +3026,64 @@
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
-          <t>data/papers/</t>
+          <t>lib_sterics.py</t>
         </is>
       </c>
     </row>
     <row r="31" ht="108" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>WT MD baseline / loop dynamics</t>
+          <t>MM-GBSA rescoring</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>Pocket - energetics</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Explicit-solvent MD (ff19SB/OPC, 0.15 M KCl, 2 fs, 300 ns) with a two-reference projection: fit on the rigid core, then measure gate/latch RMSD to BOTH open and closed crystals.</t>
+          <t>Replaces ref2015's pairwise Lazaridis-Karplus solvation with generalised Born: dG_bind = G_complex - G_receptor - G_ligand, averaged over an MD ensemble. ff14SB + GAFF2/AM1-BCC, igb=8, 0.15 M salt. Rosetta builds structures and never scores them.</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>Asked whether open and closed states are separable and whether MD can filter designs.</t>
+          <t>Direct attack on the diagnosed cause of the K59 failure.</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>S1 apo-open (3K3K A), S2 holo-closed (3QN1 A + ABA), S3 dimer, S4 ternary (+HAB1, Mn2+); 12 trajectories</t>
+          <t>Mandipropamid vs ABA; 7 variants x 2 arms x 100-frame ensembles</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Aug 10 - Aug 18</t>
+          <t>Aug 19</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Neither state ever converts in 1.8 us aggregate. Replicate-mean gap 5.57 A at the gate, stable at every discard from 0-150 ns. RMSF ladder: gate 3.05 open -&gt; 1.39 closed -&gt; 0.81 ternary.</t>
+          <t>⚠ THE K59 FLIP IS RETRACTED (README 40). It was an artefact of an UNCONVERGED reference: the WT-ABA complex moves +7.75 kcal/mol between 50 and 250 ps and is still drifting. Recomputed at 250 ps the pre-registered test gives the OPPOSITE answer, selectivity -8.58 (PASS) -&gt; +1.31 (FAIL). Sign-based verdicts from this method are void at these lengths; rank-based ones survive but are marginal (p = 0.049) and bounded by a 1.05 kcal/mol per-variant drift, the size of the spacing being ranked. README 42-43 retire it: +-3.85 needs n=60/variant, about 1748 GPU-hours.</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Licenses a STABILITY filter only (gate RMSD-to-closed, 3.5-4.0 A) and is BLIND to switchability - the likelier failure for an enlarged pocket. The latch fails as an RMSF filter (ratio inverts).</t>
+          <t>Ensembles only 50 ps (GBn2 runs ~380 steps/min here; pmemd no faster). The ligand-swap difference is dominated by DAMAGE TO THE ABA COMPLEX, not gain for mandipropamid. F108A comes out NULL because relaxation absorbs the clash it exists to relieve.</t>
         </is>
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>Never read a stable closed trajectory as a working switch. Inference is at replicate level: autocorrelation times 3.4-44.9 ns, so each 300 ns run holds only 3-35 independent samples.</t>
-        </is>
-      </c>
-      <c r="J31" s="9" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
+          <t>Changing the solvation model does what no sampler could - the desolvation diagnosis was right AND actionable. Also: my first error bars were fabricated (8 'independent' repacks came out byte-identical).</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>RETIRED</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3009,62 +3093,62 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>CPU cutlerlab, 14 tasks</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>58-60; jobs 27333712, 27545237</t>
+          <t>75, 75b-e; jobs 27561665, 27568930, 27569546</t>
         </is>
       </c>
     </row>
     <row r="32" ht="108" customHeight="1">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Apo-closed protomer analysis</t>
+          <t>Coumarin focused-library benchmark</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>Pocket - benchmark</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Re-analysis of the S3 mixed dimer, whose chain B is a closed, ligand-shaped protomer simulated with the ABA stripped.</t>
+          <t>Extracts the exact per-position residue menus Tian et al. built for each focused library, then measures what a method must add over a ligand-blind baseline.</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Filled the missing cell of the factorial using data already on disk.</t>
+          <t>Asked whether round-1 screening could have been skipped computationally.</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>3K3K chain B (closed, was ABA-bound), 3 x 300 ns</t>
+          <t>LIBRARY DESIGNS, not structures: Tian sd04 per-position residue menus for the Coumarin, PFAS and TNTv1/v2 focused libraries, plus 692 characterised sensor clones (sequences).</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Aug 18</t>
+          <t>Aug 14</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>Apo-closed does NOT open: zero crossings, drift -0.07 A, and the MOST RIGID gate of all 15 units (RMSF 0.72 A vs 1.39 with ABA).</t>
+          <t>Reframed the task. POSITIONS are near ligand-independent: Coumarin/PFAS/TNTv2 share 9 of their 11-14 positions, so naming the shared nine scores 82% recall with ZERO ligand information. SUBSTITUTIONS are ligand-specific: mean 3-way Jaccard 0.02.</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Confounded by the dimer, which alone drops the open gate 3.05 -&gt; 1.07 A - larger than the ligand effect being measured.</t>
+          <t>I initially claimed the coumarin library design was missing from the supplement. It was not - a column header truncated at 20 characters.</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>The stability filter is CONFORMATION-reporting, not ligand-reporting: a good gate-RMSD score carries no evidence about occupancy. Also: 3K3K is a MIXED dimer, and the name S3_apo_dimer had outranked four records saying so.</t>
-        </is>
-      </c>
-      <c r="J32" s="9" t="inlineStr">
+          <t>Predict MENUS, not positions. Focusing buys ~16 orders of magnitude (3.8e21 -&gt; 1.4e5).</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -3076,62 +3160,62 @@
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>CPU local</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>58-60; job 27545237</t>
+          <t>62_coumarin_ground_truth.py</t>
         </is>
       </c>
     </row>
     <row r="33" ht="108" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>191-residue rebuild pipeline</t>
+          <t>Beltran cannabinoid sensor table</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>MD - structure</t>
+          <t>Pocket - benchmark</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Biopython graft + PyRosetta rebuild of the complete 191-aa sequence with no chain breaks, seeded and byte-reproducible, with identity and provenance assertions at every step.</t>
+          <t>45 experimentally validated sensors across 12 cannabinoids, with mutation sets and a graded dose-response (1e4 -&gt; 10 nM).</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Removed the gapped-receptor confound from every future MD system.</t>
+          <t>A second, harder ground truth with an ORDER to recover, not just a set.</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>3K3K A/B, 3QN1 A; ABA</t>
+          <t>Sensor SEQUENCE table (no solved structures): 45 PYR1 variants vs WIN 55,212-2, the JWH series, D9-THC, CBDA, CP 47,497. WIN 55,212-2 is an aminoalkylindole synthetic cannabinoid, so it belongs in this set despite the name looking unlike the others.</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Aug 17</t>
+          <t>Aug 18-19</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>7 verified structures; every chain 191 residues, 0 peptide-bond breaks, 0 clashes, ligand-lining side chains unmoved to 0.000 A.</t>
+          <t>Extracted in full. A160 mutated in 38/45, Y120 in 33/45, F159 in 24/45. Ligand-specific signal sits at K59 (Q/N/S/T/A/R), H115Q, V83, E141, V164, V81.</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Cost two structural defects before the cause was found - a 0.36 A inter-chain clash and K59 collapsing 2.85 -&gt; 1.68 A into an empty cavity.</t>
+          <t>Even more position-saturated than coumarin; substitutions reused within a chemical family (A160G 27x, Y120G 23x). Nine substitutions sit OUTSIDE the 5 A pocket - PYR1-WIN gets its last order of magnitude from E4G.</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>FastRelax.set_movemap() restricts MINIMISATION only; repacking needs a TaskFactory or the whole pose is repacked. Backbone RMSD reported 0.000 A throughout - always check side chains and inter-chain contacts.</t>
-        </is>
-      </c>
-      <c r="J33" s="9" t="inlineStr">
+          <t>A graded sensitivity ladder is a far stronger benchmark than a hit list. K59Q/K59N are neutral, so they should be reachable where K59R was not - a free sanity check.</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
         <is>
           <t>ACTIVE</t>
         </is>
@@ -3148,81 +3232,81 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>67, 67c, 68; lib_resnumber/structqc/rosetta</t>
+          <t>data/beltran/win_sensors.json</t>
         </is>
       </c>
     </row>
     <row r="34" ht="108" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Conformation x occupancy factorial</t>
+          <t>Literature protocol review</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>Pocket - benchmark</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>The 2x2 that README 19b set up and only ever filled on the diagonal: open/closed x apo/holo, all four cells on ONE build protocol.</t>
+          <t>Read six papers from their Methods sections, not abstracts, to establish what the field does and what the honest baseline is.</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Separates 'the gate holds its shape' from 'the ligand holds the gate'.</t>
+          <t>Calibrated our results against published practice before investing further.</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>S1 open+apo, S2 closed+ABA, S9 closed+apo, S10 open+ABA (ABA transplanted, backbone bit-identical)</t>
+          <t>Six papers (PDFs + extracted Methods text): Leonard 2026, An 2024, Tian 2025, Park 2023, ACS Chem Biol 2024, Nat Biotech 2026.</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Aug 18 - running</t>
+          <t>Aug 19</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
         <is>
-          <t>S10 (open + ABA) never existed before and is now built and verified. 5 of 12 replicates complete, including both S10 reps 0 and 2.</t>
+          <t>Leonard's 'dock to sequence' MUTATES WT to a known weak-hit sequence before placing any pose - their method improves a known weak binder and cannot start from a ligand alone. An et al. picked cutoffs by MANUAL INSPECTION. RbsB precedent: 2M variants screened for 1.2-1.5x induction.</t>
         </is>
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Not yet analysed. The old-tree S9 could not be reused: it is KCl where S1/S2 are NaCl, which would put a cation swap inside the key comparison.</t>
+          <t>Leonard hard-filters on an H-bond to the latch water, which mandipropamid misses by 5.07-5.19 A - their protocol would reject the correct pose.</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>Gate closure on ligand binding is the one arm where the barrier is plausibly downhill - pre-registered so 'nothing happened' cannot later be written up as 'ABA does not close the gate'.</t>
-        </is>
-      </c>
-      <c r="J34" s="11" t="inlineStr">
-        <is>
-          <t>ACTIVE (running)</t>
+          <t>The field's baseline is low, and our benchmark is strictly harder than Leonard's. The ACS Chem Biol paper independently confirmed R79 H-bonds F52's carbonyl at &gt;90% occupancy, explaining one of our control failures from the other direction.</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>now</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>GPU</t>
+          <t>local</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr">
         <is>
-          <t>69, 69b, 70; job 27547457</t>
+          <t>data/papers/</t>
         </is>
       </c>
     </row>
     <row r="35" ht="108" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Non-cognate ligand MD (S6-S8)</t>
+          <t>WT MD baseline / loop dynamics</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -3232,47 +3316,47 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Same closed receptor, three ABA-sized ligands from three chemical classes, three docked poses each.</t>
+          <t>Explicit-solvent MD (ff19SB/OPC, 0.15 M KCl, 2 fs, 300 ns) with a two-reference projection: fit on the rigid core, then measure gate/latch RMSD to BOTH open and closed crystals.</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Designed to test whether the stability filter can rank LIGANDS or only conformations.</t>
+          <t>Asked whether open and closed states are separable and whether MD can filter designs.</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Imperatorin, Flutamide, alpha-Estradiol (19-20 heavy atoms, MW 270-276) in WT closed PYR1</t>
+          <t>S1 apo-open (3K3K A), S2 holo-closed (3QN1 A + ABA), S3 dimer, S4 ternary (+HAB1, Mn2+); 12 trajectories</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Aug 14 (built)</t>
+          <t>Aug 10 - Aug 18</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Built and pose-verified; three replicates per ligand start from three DIFFERENT poses, so pose sensitivity is measured rather than assumed.</t>
+          <t>Neither state ever converts in 1.8 us aggregate. Replicate-mean gap 5.57 A at the gate, stable at every discard from 0-150 ns. RMSF ladder: gate 3.05 open -&gt; 1.39 closed -&gt; 0.81 ternary.</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>Never submitted. Partly superseded by the apo-closed result, which answered the same question more cheaply.</t>
+          <t>Licenses a STABILITY filter only (gate RMSD-to-closed, 3.5-4.0 A) and is BLIND to switchability - the likelier failure for an enlarged pocket. The latch fails as an RMSF filter (ratio inverts).</t>
         </is>
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>Absence of ligand release is NOT evidence of binding - residence times are us-ms and 300 ns cannot sample unbinding.</t>
-        </is>
-      </c>
-      <c r="J35" s="12" t="inlineStr">
-        <is>
-          <t>PLANNED</t>
+          <t>Never read a stable closed trajectory as a working switch. Inference is at replicate level: autocorrelation times 3.4-44.9 ns, so each 300 ns run holds only 3-35 independent samples.</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
         <is>
-          <t>P2 - after the factorial</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
@@ -3282,79 +3366,347 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>63-66</t>
+          <t>58-60; jobs 27333712, 27545237</t>
         </is>
       </c>
     </row>
     <row r="36" ht="108" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
+          <t>Apo-closed protomer analysis</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Re-analysis of the S3 mixed dimer, whose chain B is a closed, ligand-shaped protomer simulated with the ABA stripped.</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Filled the missing cell of the factorial using data already on disk.</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>3K3K chain B (closed, was ABA-bound), 3 x 300 ns</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Aug 18</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>Apo-closed does NOT open: zero crossings, drift -0.07 A, and the MOST RIGID gate of all 15 units (RMSF 0.72 A vs 1.39 with ABA).</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Confounded by the dimer, which alone drops the open gate 3.05 -&gt; 1.07 A - larger than the ligand effect being measured.</t>
+        </is>
+      </c>
+      <c r="I36" s="7" t="inlineStr">
+        <is>
+          <t>The stability filter is CONFORMATION-reporting, not ligand-reporting: a good gate-RMSD score carries no evidence about occupancy. Also: 3K3K is a MIXED dimer, and the name S3_apo_dimer had outranked four records saying so.</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L36" s="7" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>58-60; job 27545237</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="108" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>191-residue rebuild pipeline</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>MD - structure</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Biopython graft + PyRosetta rebuild of the complete 191-aa sequence with no chain breaks, seeded and byte-reproducible, with identity and provenance assertions at every step.</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Removed the gapped-receptor confound from every future MD system.</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>3K3K A/B, 3QN1 A; ABA</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Aug 17</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>7 verified structures; every chain 191 residues, 0 peptide-bond breaks, 0 clashes, ligand-lining side chains unmoved to 0.000 A.</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Cost two structural defects before the cause was found - a 0.36 A inter-chain clash and K59 collapsing 2.85 -&gt; 1.68 A into an empty cavity.</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>FastRelax.set_movemap() restricts MINIMISATION only; repacking needs a TaskFactory or the whole pose is repacked. Backbone RMSD reported 0.000 A throughout - always check side chains and inter-chain contacts.</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>CPU local</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>67, 67c, 68; lib_resnumber/structqc/rosetta</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="108" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Conformation x occupancy factorial</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>The 2x2 that README 19b set up and only ever filled on the diagonal: open/closed x apo/holo, all four cells on ONE build protocol.</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Separates 'the gate holds its shape' from 'the ligand holds the gate'.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>S1 open+apo, S2 closed+ABA, S9 closed+apo, S10 open+ABA (ABA transplanted, backbone bit-identical)</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Aug 18 - running</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>S10 (open + ABA) never existed before and is now built and verified. 5 of 12 replicates complete, including both S10 reps 0 and 2.</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Not yet analysed. The old-tree S9 could not be reused: it is KCl where S1/S2 are NaCl, which would put a cation swap inside the key comparison.</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
+        <is>
+          <t>Gate closure on ligand binding is the one arm where the barrier is plausibly downhill - pre-registered so 'nothing happened' cannot later be written up as 'ABA does not close the gate'.</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>ACTIVE (running)</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>now</t>
+        </is>
+      </c>
+      <c r="L38" s="7" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>69, 69b, 70; job 27547457</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="108" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Non-cognate ligand MD (S6-S8)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Same closed receptor, three ABA-sized ligands from three chemical classes, three docked poses each.</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Designed to test whether the stability filter can rank LIGANDS or only conformations.</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Imperatorin, Flutamide, alpha-Estradiol (19-20 heavy atoms, MW 270-276) in WT closed PYR1</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Aug 14 (built)</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Built and pose-verified; three replicates per ligand start from three DIFFERENT poses, so pose sensitivity is measured rather than assumed.</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Never submitted. Partly superseded by the apo-closed result, which answered the same question more cheaply.</t>
+        </is>
+      </c>
+      <c r="I39" s="7" t="inlineStr">
+        <is>
+          <t>Absence of ligand release is NOT evidence of binding - residence times are us-ms and 300 ns cannot sample unbinding.</t>
+        </is>
+      </c>
+      <c r="J39" s="12" t="inlineStr">
+        <is>
+          <t>PLANNED</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>P2 - after the factorial</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>GPU</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>63-66</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="108" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>ABA enantiomer / non-cognate controls</t>
         </is>
       </c>
-      <c r="B36" s="7" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="C36" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>Isosteric control: (-)-ABA is identical in formula, bulk and parameters, differing only in chirality, so any difference is chemistry rather than size.</t>
         </is>
       </c>
-      <c r="D36" s="7" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Requested, to test whether gate behaviour is ligand-specific.</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E40" s="7" t="inlineStr">
         <is>
           <t>(-)-ABA plus an unrelated matched molecule; WT PYR1</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
+      <c r="F40" s="7" t="inlineStr">
         <is>
           <t>planned</t>
         </is>
       </c>
-      <c r="G36" s="7" t="inlineStr">
+      <c r="G40" s="7" t="inlineStr">
         <is>
           <t>Not yet run.</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H40" s="7" t="inlineStr">
         <is>
           <t>Must NOT be read as a gate-opening test: nothing opens on this timescale in any of 15 units. The graded RMSF ladder is the observable that responds to ligand.</t>
         </is>
       </c>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="I40" s="7" t="inlineStr">
         <is>
           <t>Phaseic acid would add a third rung, turning a binary contrast into a graded ladder that is much harder to explain away.</t>
         </is>
       </c>
-      <c r="J36" s="12" t="inlineStr">
+      <c r="J40" s="12" t="inlineStr">
         <is>
           <t>PLANNED</t>
         </is>
       </c>
-      <c r="K36" s="7" t="inlineStr">
+      <c r="K40" s="7" t="inlineStr">
         <is>
           <t>P2 - after the factorial</t>
         </is>
       </c>
-      <c r="L36" s="7" t="inlineStr">
+      <c r="L40" s="7" t="inlineStr">
         <is>
           <t>GPU</t>
         </is>
       </c>
-      <c r="M36" s="7" t="inlineStr">
+      <c r="M40" s="7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M36"/>
+  <autoFilter ref="A1:M40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>